<commit_message>
de actualiza formato de asistencia
</commit_message>
<xml_diff>
--- a/assets/documentos/L-RF-14-2026 Lista de Asistencia.xlsx
+++ b/assets/documentos/L-RF-14-2026 Lista de Asistencia.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amendozat\Desktop\DIGITAL\respaldo intranet\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amendozat\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03A69997-BE7E-4EF5-B5F7-AB753B0C6BB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B01112B-7A52-4E40-8845-BB58593B7EC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>(Folio Tramite: GRC, PT, GO)</t>
   </si>
@@ -84,6 +84,19 @@
   </si>
   <si>
     <t>NOMBRE COMPLETO, PUESTO Y FIRMA DEL RESPONSABLE</t>
+  </si>
+  <si>
+    <r>
+      <t>Aviso de Privacidad:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13.5"/>
+        <rFont val="Arial Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> La Secretaría de Turismo e Identidad del Estado de Guanajuato, se obliga a proteger y tratar los datos personales recabados, en términos de lo previsto por la Ley de Protección de Datos Personales en Posesión de Sujetos Obligados para el Estado de Guanajuato y demás normatividad aplicable. La confidencialidad de los datos está garantizada y los mismos están protegidos. Únicamente las personas autorizadas tendrán acceso a sus datos.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -93,7 +106,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -145,6 +158,17 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="13.5"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13.5"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -348,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -406,6 +430,12 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -439,11 +469,11 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -807,7 +837,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:J36"/>
+  <dimension ref="B1:J38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.42578125" customWidth="1"/>
@@ -845,12 +875,12 @@
     </row>
     <row r="4" spans="2:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="1"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="40"/>
-      <c r="F4" s="40"/>
-      <c r="G4" s="40"/>
-      <c r="H4" s="40"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="29"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="29"/>
       <c r="I4" s="2"/>
     </row>
     <row r="5" spans="2:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -887,101 +917,101 @@
     </row>
     <row r="8" spans="2:10" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="1"/>
-      <c r="C8" s="41" t="s">
+      <c r="C8" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="41"/>
-      <c r="E8" s="41"/>
-      <c r="F8" s="41"/>
-      <c r="G8" s="41"/>
-      <c r="H8" s="41"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
       <c r="I8" s="2"/>
     </row>
     <row r="9" spans="2:10" s="9" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="7"/>
-      <c r="C9" s="33" t="s">
+      <c r="C9" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="34"/>
-      <c r="E9" s="34"/>
-      <c r="F9" s="35"/>
-      <c r="G9" s="30" t="s">
+      <c r="D9" s="36"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="H9" s="32"/>
+      <c r="H9" s="34"/>
       <c r="I9" s="8"/>
       <c r="J9" s="10"/>
     </row>
     <row r="10" spans="2:10" s="9" customFormat="1" ht="28.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="7"/>
-      <c r="C10" s="30" t="s">
+      <c r="C10" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="31"/>
-      <c r="E10" s="31"/>
-      <c r="F10" s="31"/>
-      <c r="G10" s="31"/>
-      <c r="H10" s="32"/>
+      <c r="D10" s="33"/>
+      <c r="E10" s="33"/>
+      <c r="F10" s="33"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="34"/>
       <c r="I10" s="8"/>
       <c r="J10" s="10"/>
     </row>
     <row r="11" spans="2:10" s="9" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="7"/>
-      <c r="C11" s="33" t="s">
+      <c r="C11" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="35" t="s">
+      <c r="D11" s="37" t="s">
         <v>0</v>
       </c>
       <c r="E11" s="28"/>
-      <c r="F11" s="30" t="s">
+      <c r="F11" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="G11" s="31"/>
-      <c r="H11" s="32"/>
+      <c r="G11" s="33"/>
+      <c r="H11" s="34"/>
       <c r="I11" s="8"/>
       <c r="J11" s="11"/>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B12" s="1"/>
-      <c r="C12" s="37"/>
-      <c r="D12" s="37"/>
-      <c r="E12" s="37"/>
-      <c r="F12" s="37"/>
-      <c r="G12" s="37"/>
-      <c r="H12" s="37"/>
+      <c r="C12" s="39"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="39"/>
+      <c r="F12" s="39"/>
+      <c r="G12" s="39"/>
+      <c r="H12" s="39"/>
       <c r="I12" s="2"/>
     </row>
     <row r="13" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="1"/>
-      <c r="C13" s="36" t="s">
+      <c r="C13" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="D13" s="36" t="s">
+      <c r="D13" s="38" t="s">
         <v>2</v>
       </c>
-      <c r="E13" s="38" t="s">
+      <c r="E13" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="F13" s="36" t="s">
+      <c r="F13" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="G13" s="36" t="s">
+      <c r="G13" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="H13" s="36" t="s">
+      <c r="H13" s="38" t="s">
         <v>4</v>
       </c>
       <c r="I13" s="2"/>
     </row>
     <row r="14" spans="2:10" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="1"/>
-      <c r="C14" s="36"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="39"/>
-      <c r="F14" s="36"/>
-      <c r="G14" s="36"/>
-      <c r="H14" s="36"/>
+      <c r="C14" s="38"/>
+      <c r="D14" s="38"/>
+      <c r="E14" s="41"/>
+      <c r="F14" s="38"/>
+      <c r="G14" s="38"/>
+      <c r="H14" s="38"/>
       <c r="I14" s="2"/>
     </row>
     <row r="15" spans="2:10" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1212,10 +1242,10 @@
       <c r="D34" s="13"/>
       <c r="E34" s="13"/>
       <c r="F34" s="22"/>
-      <c r="G34" s="29" t="s">
+      <c r="G34" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="H34" s="29"/>
+      <c r="H34" s="31"/>
       <c r="I34" s="2"/>
     </row>
     <row r="35" spans="2:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
@@ -1228,9 +1258,35 @@
       <c r="H35" s="17"/>
       <c r="I35" s="4"/>
     </row>
-    <row r="36" spans="2:9" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="36" spans="2:9" ht="18" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="C36" s="42" t="s">
+        <v>16</v>
+      </c>
+      <c r="D36" s="42"/>
+      <c r="E36" s="42"/>
+      <c r="F36" s="42"/>
+      <c r="G36" s="42"/>
+      <c r="H36" s="42"/>
+    </row>
+    <row r="37" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="C37" s="43"/>
+      <c r="D37" s="43"/>
+      <c r="E37" s="43"/>
+      <c r="F37" s="43"/>
+      <c r="G37" s="43"/>
+      <c r="H37" s="43"/>
+    </row>
+    <row r="38" spans="2:9" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C38" s="43"/>
+      <c r="D38" s="43"/>
+      <c r="E38" s="43"/>
+      <c r="F38" s="43"/>
+      <c r="G38" s="43"/>
+      <c r="H38" s="43"/>
+    </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
+    <mergeCell ref="C36:H38"/>
     <mergeCell ref="C4:H4"/>
     <mergeCell ref="C8:H8"/>
     <mergeCell ref="G34:H34"/>

</xml_diff>